<commit_message>
Support official website analysis in intake workflow
</commit_message>
<xml_diff>
--- a/assets/simple-feed-template.xlsx
+++ b/assets/simple-feed-template.xlsx
@@ -39,7 +39,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +60,9 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D9EAF7"/>
       </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid"/>
     </fill>
   </fills>
   <borders count="2">
@@ -88,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -100,6 +103,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -467,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -710,7 +716,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>地址、电话、WhatsApp是什么？</t>
+          <t>官网或线上店铺是什么？</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
@@ -721,7 +727,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>必填</t>
+          <t>建议</t>
         </is>
       </c>
     </row>
@@ -733,32 +739,56 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>有哪些照片、证书、授权？</t>
+          <t>地址、电话、WhatsApp是什么？</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr"/>
       <c r="D13" s="4" t="inlineStr">
         <is>
+          <t>企业背景、推广转化</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>必填</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>有哪些照片、证书、授权？</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
           <t>企业背景、信任背书</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>必填</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>推广就绪判断：公司名、地址/电话/WhatsApp、产品服务、3 个优势、1-3 个案例、照片/授权齐全后，即可展开成九大单元用于推广。</t>
+    <row r="15" ht="40" customHeight="1"/>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>推广就绪判断：公司名、官网/线上店铺、地址/电话/WhatsApp、产品服务、3 个优势、1-3 个案例、照片/授权齐全后，即可展开成九大单元用于推广。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -771,7 +801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -933,39 +963,57 @@
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>9. 地址/电话/WhatsApp</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>9. 官网/线上店铺</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>企业背景、推广转化</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>无法核实官网或线上渠道，企业可信度和转化入口缺失</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="38" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>10. 地址/电话/WhatsApp</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>企业背景、推广转化</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>客户看到内容也无法联系成交</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="38" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>10. 照片/证书/授权</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>11. 照片/证书/授权</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>企业背景、信任背书</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>信任感不足，平台审核和收录可能受影响</t>
         </is>
       </c>
     </row>
+    <row r="13"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -977,7 +1025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1068,6 +1116,18 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>官网来源</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>客户提供官网或线上店铺时，先抓取并分析官网内容，再把可核验信息用于九大单元；不可访问或不确定时不编造。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>